<commit_message>
Add ACLED-confirmed spellings for third labelling pass; flag genuine ambiguity
Resolver additions from Samuel's third pass (77 rows labelled): Maxaas confirmed
against ACLED as Bulo Burto; Brava, Khada, the Galkayu/Jamaame east-west splits,
Zeila, Buleburte and Dusamreb added as straightforward spelling variants.

Ceel Garas is deliberately left unmapped. ACLED itself files it under two
different districts (Dhuusamareeb and Xudur) depending on the report, so it
cannot be resolved without reading the specific source; auto-mapping it to
either would corrupt ground truth. It now reports as unresolved rather than
guessed, alongside a handful of place names (Bargaal, Hafun, Guriel, Rako,
Ufeyn and others) not found in any source in this repository and left for
Samuel to confirm from firsthand knowledge of the report.
</commit_message>
<xml_diff>
--- a/data/geoparser_validation/geoparser_labelling_workbook.xlsx
+++ b/data/geoparser_validation/geoparser_labelling_workbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samue\OneDrive\Desktop\Msc Data Science\Dissertation\Geoparser verification\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C784190A-EABB-4CDC-91F4-AF486FAA1DA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{670AD2FD-D41A-424F-BEF6-452A9DB33148}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1389" uniqueCount="873">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1488" uniqueCount="911">
   <si>
     <t>ReliefWeb geoparser validation: labelling instructions</t>
   </si>
@@ -3127,12 +3127,6 @@
     <t>Afgoye;Beletweyn;Buur Xakaba;Bossaso;Balcad</t>
   </si>
   <si>
-    <t>Bossaso; Balad; Garowe; Burhakabo; Gardo; Daynile (Mogadishu-Daynile); Mahaday; Mudug; Karkaar; Bay (Baydhaba/Baidoa); Gedo; Lower Juba (Kismaayo/Kismayo); Luuq; Doolow; Qoryooley; Xudun; Diinsoor; Borama; Cadaado; Jariiban; Laas Caanood; Mogadishu-Kaxda</t>
-  </si>
-  <si>
-    <t>Mogadishu-Wadajir; Mogadishu-Waaberi; Mogadishu-Abdiaziz; Ceel Waaq; Garbahaarey; Hargeysa; Berbera; Afmadow; Jamaame; Marka; Wanla Weyn; Xudur; Banadir; Galgadud; Mudug G; Hiiraan; Middle Shebelle; Lower Shabelle; Middle Juba; Ayn; Bari; Gardafuu; Nugaal; Sanaag; Sool; Bakool</t>
-  </si>
-  <si>
     <t>BAY</t>
   </si>
   <si>
@@ -3140,9 +3134,6 @@
   </si>
   <si>
     <t>Adan Yabal; Afgooye; Afmadow; Badhaadhe; Balcad; Bandarbeyla; Baraawe; Bardheere; Baydhaba; Belet Xaawo; Beletweyne; Berbera; Bondhere; Borama; Bossaso; Bulo Burto; Burco; Burtinle; Buuhoodle; Buur Hakaba; Bu'aale; Cabudwaaq; Cadaado; Cadale; Caluula; Caynabo; Ceel Afweyn; Ceel Barde; Ceel Buur; Ceel Dheer; Ceel Waaq; Ceerigaabo; Dayniile; Dharkenley; Dhuusamareeb; Diinsoor; Doolow; Eyl; Gaalkacyo; Garbaharey; Garoowe; Gebiley; Heliwa; Hobyo; Hodan; Iskushuban; Jalalaqsi; Jamaame; Jariiban; Jilib; Jowhar; Kismaayo; Kurtunwaarey; Laas Caanood; Laasqoray; Lughaye; Luuq; Marka; Owdweyne; Qandala; Qansax Dheere; Qardho; Qoryooley; Rabdhuree; Saakow; Sablaale; Shangani; Sheikh; Shibis; Taleex; Tayeeglow; Waajid; Wadajir; Wanla Weyn; Wardhigley; Xarardheere; Xudun; Xuduur; Yaaqshid; Zeylac</t>
-  </si>
-  <si>
-    <t>Baidoa; Balcad; Banadir; Buuhoodle; Jowhar; Kismayo; Laas Caanood; Luuq</t>
   </si>
   <si>
     <t>Data type: report</t>
@@ -3212,12 +3203,6 @@
     <t>Banadir;Baydhaba;Afgooye;Doolow;Dhobley</t>
   </si>
   <si>
-    <t>Afgoye; Baidoa; Balad (Hawadley Village); Banadir; Beletweyne; Borama; Bosaso; Bulo Burte; Burao; Burhakabe; Danyile; Dhahar; Garowe; Jalalaqsi; Jowhar; Kismayo; Kuntunwarey; Mahaday; Merka; Qardho; South Galkacyo</t>
-  </si>
-  <si>
-    <t>Abdul Aziz; Badhan; Barawe; Belethawo; Bondere; Dharkenly; Erigavo; Gabiley; Hamar jajab; Hamar weyn; Hargeisa; Hawl Wadag; Heliwa; Hodan; Kahda; Karan; Lasqoray; Owdweyne; Qoryoley; Shangani; Shibis; Waberi; Wadajir; Wardegley; Yaqshid</t>
-  </si>
-  <si>
     <t>Afmadow; Baardheere; Badhaadhe; Ceelwaaq; Dhobley; Dollow; Kismayo</t>
   </si>
   <si>
@@ -3274,6 +3259,135 @@
   </si>
   <si>
     <t>Abdul Aziz; Badhan; Badhan SL; Barawe; Belethawo; Bondere; Burao; Danyile; Dhahar SL; Dharkenly; Eigavo; Erigavo; Gabiley; Hamar jajab; Hamar weyn; Hargeisa; Hawl Wadag; Heliwa; Hodan; Kahda; Karan; Kurtunwaray; Lasqoray; Owdweyne; Qoryoley; Shangani; Shibis; South Galkacyo; South Galkaio; Waberi; Wadajir; Wardegley; Yaqshid</t>
+  </si>
+  <si>
+    <t>Data type: Infographic</t>
+  </si>
+  <si>
+    <t>Aadan Yabaal (Aden Yabaal); Afgooye; Afmadow; Baardheere; Badhaadhe; Balcad; Bandarbeyla; Baraawe; Baydhaba (Baidoa); Belet Weyne; Belet Xaawo; Berbera; Boorama (Borama); Bossaso; Bualle; Bulo Burte; Burco (Burao); Burtinle; Buuhoodle; Buur Hakaba (Burhakaba); Cabudwaaq; Cadale; Cadaado; Caluula; Caynabo; Ceel Afweyn; Ceel Barde; Ceel Buur; Ceel Dheer; Ceel Waaq; Ceerigaabo; Diinsoor; Doolow; Dhuusamarreeb; Eyl; Gaalkacyo; Galdogob; Garbahaarey; Garowe; Gebiley; Hargeysa; Hobyo; Iskushuban; Jalalaqsi; Jamaame; Jariiban; Jilib; Jowhar; Kismaayo (Kismayo); Kurtunwaarey; Laas Caanood; Laasqoray; Lughaye; Luuq; Mahaday; Marka; Oodweyne; Qandala; Qardho; Qoryooley; Rab Dhuure; Saakow; Sablaale; Taleex; Tiyeeglow (Tijieglo); Waajid; Wanla Weyn; Xarardheere; Xudur; Xudun; Zeylac</t>
+  </si>
+  <si>
+    <t>Afgooye; Afmadow; Baardheere; Badhaadhe; Baki; Bandarbeyla; Baraawe; Baydhaba; Belet Weyne; Belet Xaawo; Berbera; Borama; Bualle; Buhoodle; Bulo Burte; Burco; Burtinle; Buur Hakaba; Cabudwaaq; Cadaado; Caluula; Carmo; Ceel Afweyn; Ceel Barde; Ceel Waaq; Ceerigaabo; Dhahar; Dinsoor; Dollow; Eyl; Gaalkacyo; Garbahaarey; Gebiley; Hargeisa; Hobyo; Iskushuban; Jowhar; Kismaayo; Kurtunwaarey; Laas Canood; Laasqoray; Lughaye; Luuq; Marka; Mataban; Owdweyne; Qandala; Qansadheere; Qardho; Qoryooley; Rab Dhuure; Saakow; Sablaale; Sheikh; Taleex; Tayeeglow; Waajid; Wanla Weyne; Xudur; Xudun; Zeylac</t>
+  </si>
+  <si>
+    <t>Data type: News and press releases</t>
+  </si>
+  <si>
+    <t>Banadir, Puntland, South-West, Jubaland, and Hirshabelle</t>
+  </si>
+  <si>
+    <t>Baidoa (Baydhabo); Dhusamareeb; Gaalkacyo; Garowe; Hargeisa; Jamaame (Jamame); Jowhar; Kismayo; Mogadishu,Beledweyne</t>
+  </si>
+  <si>
+    <t>report</t>
+  </si>
+  <si>
+    <t>Baidoa; Daynile; Dhuusamarreeb; Gaalkacyo; Garowe; Hobyo; Jariiban; Khada; Xarardheere</t>
+  </si>
+  <si>
+    <t>Abdiaziz; Bondhere; Dharkenley; Hamar Jajab; Hamar Weyne; Hodan; Howlwadaag; Huriwa (Heliwa); Karan; Shangani; Shibis; Waberi; Wadajir; Warta Nabada; Yaqshid</t>
+  </si>
+  <si>
+    <t>map</t>
+  </si>
+  <si>
+    <t>Cabudwaaq; Cadaado; Ceel Buur; Ceel Dheer; Dhuusamarreeb</t>
+  </si>
+  <si>
+    <t>Adan Yabaal; Belet Weyne; Bulo Burto; Cadale; Gaalkacyo; Hobyo; Jalalaqsi; Mahas; Mataban; Xarardheere</t>
+  </si>
+  <si>
+    <t>news and press release</t>
+  </si>
+  <si>
+    <t>Beledweyne; Bosaso; Garowe; Jowhar; Kismayo; Mogadishu</t>
+  </si>
+  <si>
+    <t>Baidoa; Dhusamareb; Hargeisa</t>
+  </si>
+  <si>
+    <t>Afgooye; Afmadow; Baardheere; Badhan; Baidoa; Balcad; Bandarbeyla; Belet Weyne; Belet Xaawo; Baki; Borama; Bossaso; Bu'aale; Bulo Burto; Burco; Burtinle; Buuhoodle; Cabudwaaq; Ceel Afweyn; Ceel Barde; Ceel Dheer; Daynile; Dhahar; Dhuusamarreeb; Diinsoor; Doolow; Galdogob; Gaalkacyo; Garowe; Hargeysa; Heliwa; Hobyo; Jamaame; Jariiban; Jowhar; Kaxda; Kismayo; Kurtunwaarey; Laas Caanood; Marka; Qansax Dheere; Qardho; Qoryooley; Saakow; Xudur; Xudun</t>
+  </si>
+  <si>
+    <t>Jilib; Lughaye</t>
+  </si>
+  <si>
+    <t>infographics</t>
+  </si>
+  <si>
+    <t>Baidoa; Balcad (Bal'ad); Badhan; Beledweyne; Bosaso; Bulo Burte (Buleburte); Burco; Cabudwaaq (Abudwak); Cadaado (Adado); Ceel Dheer (El-dher); Dhuusamarreeb (Dhusamareb); Gaalkacyo (Galkayo); Galdogob (Goldogob); Hargeisa; Jariiban (Jarriban); Jowhar; Karan; Kismayo; Qoryooley (Torotorow); Xarardheere</t>
+  </si>
+  <si>
+    <t>Aden Yabal (Aden Yabal / Galad / Runingod); Adado; Afmadow; Baidoa; Bardera; Bulo Burti; Burdubo; Danyile; Dinsor (Dinsor district); El Bur; El Waq; Galhareri; Galkayu North; Galkayu South; Hagar; Heliwa; Hobyo; Hodan; Jilib East; Jowhar; Kismayu (Kismayo); Las Anod; Mahas; Qanaah Dere (Qansax Dheere); Salagle; Waberi; Yaqshid</t>
+  </si>
+  <si>
+    <t>Abdul Aziz; Adale; Afgoi; Alula; Awdheegle; Aynabo; Badhadhe; Badhan; Baki; Balad; Balanbale; Baligubadle; Bargaal; Bayla (Bender Bayla); Belet Hawa; Belet Weyne; Berbera; Berdale; Bondere; Borama; Bossaso; Brava; Buhodle; Buaale; Burhakaba; Burtinle; Caluula; Canyelo; Ceel Barde (El Barde); Ceel Dhere (El Dhere); Dangoroyo; Dharkenly; Dolo; Dusamreb; El Afweyn; Elgaras; Erigavo; Eyl; Gabiley; Gardo; Garbaharey; Garowe; Gedwein; Goldogob; Guriel; Hafun; Hamar Jabjab; Hamar Weyn; Haradhere; Hargeisa; Hawal Wadag; Hudun; Iskushuban; Jalalaqsi; Jamaame East; Jamaame West; Jilib West; Kahda; Karan; Kurtunwaarey; Luuq; Lughaya; Madina; Mahaday; Marka; Mataban; Odwayne; Qandala; Qoryoley; Rabdure; Raga Elle; Rako; Sablale; Sakow; Sheikh; Taleh; Tiyeglo; Ufeyn; Waciya; Wajid; Wanleweyne; Wardegly; Warsheikh; Zeila</t>
+  </si>
+  <si>
+    <t>Adan Yabal; Afgooye; Afmadow; Baardheere (Bardheere); Badhaadhe; Baraawe; Baydhaba; Beletweyne; Bondhere; Bossaso; Bulo Burto; Burco; Buur Hakaba; Cabudwaaq; Cadale; Cadaado; Caluula; Caynabo; Ceel Afweyn; Ceel Barde (Celbarde); Ceel Buur; Ceel Dheer; Ceel Waaq; Ceerigaabo; Dayniile; Dharkenley; Dhuusamarreeb; Diinsoor; Doloow; Galkayo; Galdogob; Garowe; Hamar Jajab; Heliwa; Hobyo; Hodan; Iskushuban; Jalalaqsi; Jamaame; Jowhar; Kismaayo; Laas Caanood; Laasqoray; Luuq; Marka; Owdeweyne; Qandala; Qansax Dheere; Qoryooley; Rabdhuree; Shangani; Shibis; Talex; Waajid; Wadajir; Wanla Weyn; Wardhigley; Xarardheere; Xuduur (Xudun/Xuduur); Yaaqshid</t>
+  </si>
+  <si>
+    <t>Awdheegle; Baki; Balanbale; Baligubadle; Bandarbeyla; Berbera; Berdale; Borama; Brava; Buhoodle; Burdubo; Burtinle; Garbahaarey; Hagar; Hargeysa; Jilib; Kurtunwaarey; Lughaye; Mahaday; Mataban; Qardho; Raga Elle; Saakow; Sablaale; Salagle; Sheikh; Tayeeglow; Warsheikh; Zeila</t>
+  </si>
+  <si>
+    <t>Afgooye; Afmadow; Baardheere; Baidoa; Balcad; Belet Weyne; Dayniile; Gaalkacyo; Garoowe; Hodan; Jamaame; Jowhar; Kahda; Kismaayo; Luuq</t>
+  </si>
+  <si>
+    <t>Burco; Buuhoodle; Owdweyne; Sheikh</t>
+  </si>
+  <si>
+    <t>Berbera; Caynabo; Ceel Afweyn; Ceerigaabo; Gebiley; Hargeysa; Laas Caanood; Salahley; Xudun</t>
+  </si>
+  <si>
+    <t>Adado; Adan Yabaal; Baidoa; Bardheere; Beletweyne; Bosasso; Burco (Burao); Ceel Barde (Elberde); Dhuusamarreeb (Dhusamareb); Doolow (Dolow); Gaalkacyo (Galkacyo); Garowe; Hargeisa; Kismayo (Kismayu); Mogadishu (Banadir); Qoryooley</t>
+  </si>
+  <si>
+    <t>Baidoa; Balcad (Balad / Buurfuule); Badhan; Bardera; Beletweyne; Buleburte; Burco (Burao / Kalbare / Dhoqoshey / Bali-Hajin); Buurdhubo; Cabudwaaq (Abudwak); Cadaado (Cadado / Barleef); Ceel Dheer (El-dher / El-Ma'an); Daynile; Dhuusamarreeb (Dhusamareb / Guriel); Dollow; Gaalkacyo (Galkayo); Garadag; Huriwa; Jalalaqsi; Jowhar; Kismayo; Mahas; Xudun (Hudun</t>
+  </si>
+  <si>
+    <t>assesment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kismayo, Jamaame </t>
+  </si>
+  <si>
+    <t>Mataban, Afmadow &amp; Badhaadhe,Mogadishu</t>
+  </si>
+  <si>
+    <t>meeting minute</t>
+  </si>
+  <si>
+    <t>Ceel Buur (Elbur); Ceel Dheer (Eldheer); Gaalkacyo (Galkio); Galcad; Hobyo; Jariiban (Jariban); Xarardheere (Haradhere)</t>
+  </si>
+  <si>
+    <t>Elgaras</t>
+  </si>
+  <si>
+    <t>Adado; Aden Yabal; Afmadow; Badhadhe; Baidoa; Bardera; Beletweyne; Brava; Bulo Burti; Burdubo; Danyile; Dhuusamarreeb (Dhusamreb); El Waq; Galhareri; Galkayu North; Galkayu South; Hagar; Heliwa; Hobyo; Hodan; Jilib East; Jowhar; Karan; Kismayu (Kismayo); Las Anod; Mahas; Qansax Dheere (Qanaah Dere); Salagle; Yaqshid</t>
+  </si>
+  <si>
+    <t>Abdul Aziz; Adale; Afgoi; Alula; Awdheegle; Aynabo; Baki; Balad; Balanbale; Baligubadle; Bargaal; Bayla (Bender Bayla); Belet Hawa; Berbera; Berdale; Bondere; Borama; Bossaso; Buaale; Buhodle; Burhakaba; Burtinle; Caluula; Ceel Barde (El Barde); Ceel Dhere (El Dhere); Dangoroyo; Dharkenly; Dolo; El Afweyn; El Bur (Elbur); Elgaras; Erigavo; Eyl; Gabiley; Garbaharey; Gardo; Garowe; Goldogob; Guriel; Hafun; Hamar Jabjab; Hamar Weyn; Haradhere; Hargeisa; Hawal Wadag; Hudun; Iskushuban; Jalalaqsi; Jamaame East; Jamaame West; Jilib West; Kahda; Kurtunwaarey; Lughaya; Luuq; Madina; Mahaday; Marka; Mataban; Odwayne; Qandala; Qoryoley; Rabdure; Raga Elle; Rako; Runingod; Sablale; Sakow; Sheikh; Taleh; Tiyeglo; Ufeyn; Waciya; Wajid; Wanleweyne; Wardegly; Warsheikh; Zeila</t>
+  </si>
+  <si>
+    <t>Cadaado (Adado); Gaalkacyo (Galkayo); Hobyo; Xarardheere (Harardheere)</t>
+  </si>
+  <si>
+    <t>Baidoa; Balcad; Banadir (Mogadishu); Buuhoodle; Jowhar; Kismayo; Laas Caanood; Luuq</t>
+  </si>
+  <si>
+    <t>Gaalkacyo (Gaalkacye); Hobyo; Waajid; Xudur</t>
+  </si>
+  <si>
+    <t>Abdul Aziz; Afgoye; Badhan; Baidoa; Balad (Hawadley Village); Banadir; Barawe; Beletweyn; Belethawo; Bondere; Borama; Bosaso; Bulo Burte; Burao; Burhakabe; Danyile; Dhahar; Dharkenly; Eigavo (Erigavo); Gabiley; Gardo; Garowe; Hamar jajab; Hamar weyn; Hargeisa; Hawl Wadag; Heliwa; Hodan; Jalalaqso; Jowhar; Kahda; Karan; Kismayo; Kuntunwarey (Kurtunwaarey); Lasqoray; Mahaday; Merka; Owdweyne; Qardho; Qoryoley; Shangani; Shibis; South Galkacyo; Waberi; Wadajir; Wardegley; Yaqshid</t>
+  </si>
+  <si>
+    <t>Adan Yabaal (Aden Yabal); Afgoi; Alula; Awdheegle; Aynabo; Badhadhe; Baki; Balanbale; Baligubadle; Bargaal; Bayla; Belet Hawa; Berbera; Berdale; Brava; Buhodle; Buur Hakaba; Buurdhubo; Cabudwaaq; Cadale; Caluula; Canyelo; Ceel Afweyn; Ceel Barde; Ceel Buur; Ceel Dhere; Ceel Waaq; Dangoroyo; Dhuusamarreeb; Diinsoor; Doolow; El Bur; Galad; Galdogob; Garbaharey; Gedwein; Goldogob; Guriel; Hafun; Hagar; Haradhere; Hobyo; Hudun; Iskushuban; Jamaame; Jilib; Las Anod; Luuq; Lughaye; Mahas; Mataban; Odwayne; Qandala; Qansax Dheere; Rabdure; Raga Elle; Rako; Runingod; Saakow; Sablaale; Salagle; Sheikh; Taleh; Tiyeglo; Ufeyn; Waajid; Wanlaweyn; Warsheikh; Xudur; Zeil</t>
+  </si>
+  <si>
+    <t>Abdiaziz; Afmadow; Baidoa (Baydhaba); Berbera; Borama; Cadaado; Ceel Waaq; Daynile (Dayniile); Diinsoor; Doolow; Garbahaarey; Garowe; Hargeysa; Jamaame; Jariiban; Kaxda (Kahda); Kismayo (Kismaayo / Qamqam); Laas Caanood; Luuq; Marka; Qoryooley; Waaberi (Wadajir-Waaberi); Wadajir; Wanla Weyn; Xudun</t>
+  </si>
+  <si>
+    <t>Report</t>
   </si>
 </sst>
 </file>
@@ -4049,7 +4163,7 @@
         <v>58</v>
       </c>
       <c r="I4" s="14" t="s">
-        <v>829</v>
+        <v>827</v>
       </c>
       <c r="J4" s="9" t="s">
         <v>815</v>
@@ -4058,7 +4172,7 @@
         <v>45</v>
       </c>
       <c r="L4" s="14" t="s">
-        <v>833</v>
+        <v>830</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.45">
@@ -4094,7 +4208,7 @@
         <v>45</v>
       </c>
       <c r="L5" s="9" t="s">
-        <v>834</v>
+        <v>831</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="178.5" x14ac:dyDescent="0.45">
@@ -4170,7 +4284,7 @@
         <v>46</v>
       </c>
       <c r="L7" s="9" t="s">
-        <v>832</v>
+        <v>829</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="114.75" x14ac:dyDescent="0.45">
@@ -4208,7 +4322,7 @@
         <v>46</v>
       </c>
       <c r="L8" s="9" t="s">
-        <v>832</v>
+        <v>829</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="357" x14ac:dyDescent="0.45">
@@ -4246,7 +4360,7 @@
         <v>46</v>
       </c>
       <c r="L9" s="9" t="s">
-        <v>832</v>
+        <v>829</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="89.25" x14ac:dyDescent="0.45">
@@ -4276,13 +4390,13 @@
         <v>815</v>
       </c>
       <c r="J10" s="14" t="s">
-        <v>835</v>
+        <v>832</v>
       </c>
       <c r="K10" s="15" t="s">
         <v>46</v>
       </c>
       <c r="L10" s="14" t="s">
-        <v>836</v>
+        <v>833</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="178.5" x14ac:dyDescent="0.45">
@@ -4311,7 +4425,7 @@
         <v>84</v>
       </c>
       <c r="I11" s="9" t="s">
-        <v>837</v>
+        <v>834</v>
       </c>
       <c r="J11" s="9" t="s">
         <v>815</v>
@@ -4320,7 +4434,7 @@
         <v>45</v>
       </c>
       <c r="L11" s="14" t="s">
-        <v>838</v>
+        <v>835</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="165.75" x14ac:dyDescent="0.45">
@@ -4348,17 +4462,17 @@
       <c r="H12" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="I12" s="15" t="s">
+      <c r="I12" s="17" t="s">
         <v>818</v>
       </c>
       <c r="J12" s="17" t="s">
-        <v>839</v>
+        <v>836</v>
       </c>
       <c r="K12" s="15" t="s">
         <v>46</v>
       </c>
       <c r="L12" s="14" t="s">
-        <v>840</v>
+        <v>837</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="280.5" x14ac:dyDescent="0.45">
@@ -4387,7 +4501,7 @@
         <v>92</v>
       </c>
       <c r="I13" s="14" t="s">
-        <v>841</v>
+        <v>838</v>
       </c>
       <c r="J13" s="14" t="s">
         <v>46</v>
@@ -4396,7 +4510,7 @@
         <v>46</v>
       </c>
       <c r="L13" s="14" t="s">
-        <v>842</v>
+        <v>839</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="25.5" x14ac:dyDescent="0.45">
@@ -4470,7 +4584,7 @@
         <v>45</v>
       </c>
       <c r="L15" s="9" t="s">
-        <v>843</v>
+        <v>840</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="216.75" x14ac:dyDescent="0.45">
@@ -4508,7 +4622,7 @@
         <v>46</v>
       </c>
       <c r="L16" s="14" t="s">
-        <v>844</v>
+        <v>841</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="178.5" x14ac:dyDescent="0.45">
@@ -4537,7 +4651,7 @@
         <v>108</v>
       </c>
       <c r="I17" s="14" t="s">
-        <v>845</v>
+        <v>842</v>
       </c>
       <c r="J17" s="15" t="s">
         <v>815</v>
@@ -4575,19 +4689,19 @@
         <v>112</v>
       </c>
       <c r="I18" s="9" t="s">
-        <v>815</v>
+        <v>906</v>
       </c>
       <c r="J18" s="14" t="s">
-        <v>846</v>
+        <v>843</v>
       </c>
       <c r="K18" s="9" t="s">
         <v>46</v>
       </c>
       <c r="L18" s="14" t="s">
-        <v>842</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" ht="395.25" x14ac:dyDescent="0.45">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A19" s="7">
         <v>17</v>
       </c>
@@ -4610,11 +4724,11 @@
         <v>46</v>
       </c>
       <c r="H19" s="8"/>
-      <c r="I19" s="9" t="s">
+      <c r="I19" s="14" t="s">
+        <v>828</v>
+      </c>
+      <c r="J19" s="14" t="s">
         <v>815</v>
-      </c>
-      <c r="J19" s="14" t="s">
-        <v>830</v>
       </c>
       <c r="K19" s="9" t="s">
         <v>46</v>
@@ -4623,7 +4737,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="20" spans="1:12" ht="38.25" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:12" ht="51" x14ac:dyDescent="0.45">
       <c r="A20" s="7">
         <v>18</v>
       </c>
@@ -4646,11 +4760,11 @@
         <v>46</v>
       </c>
       <c r="H20" s="8"/>
-      <c r="I20" s="9" t="s">
+      <c r="I20" s="14" t="s">
+        <v>905</v>
+      </c>
+      <c r="J20" s="14" t="s">
         <v>815</v>
-      </c>
-      <c r="J20" s="14" t="s">
-        <v>831</v>
       </c>
       <c r="K20" s="9" t="s">
         <v>46</v>
@@ -4685,7 +4799,7 @@
         <v>122</v>
       </c>
       <c r="I21" s="14" t="s">
-        <v>848</v>
+        <v>845</v>
       </c>
       <c r="J21" s="9" t="s">
         <v>815</v>
@@ -4694,7 +4808,7 @@
         <v>46</v>
       </c>
       <c r="L21" s="14" t="s">
-        <v>847</v>
+        <v>844</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="140.25" x14ac:dyDescent="0.45">
@@ -4732,7 +4846,7 @@
         <v>46</v>
       </c>
       <c r="L22" s="9" t="s">
-        <v>849</v>
+        <v>846</v>
       </c>
     </row>
     <row r="23" spans="1:12" ht="89.25" x14ac:dyDescent="0.45">
@@ -4770,7 +4884,7 @@
         <v>46</v>
       </c>
       <c r="L23" s="9" t="s">
-        <v>849</v>
+        <v>846</v>
       </c>
     </row>
     <row r="24" spans="1:12" ht="38.25" x14ac:dyDescent="0.45">
@@ -4799,16 +4913,16 @@
         <v>134</v>
       </c>
       <c r="I24" s="14" t="s">
-        <v>850</v>
+        <v>847</v>
       </c>
       <c r="J24" s="14" t="s">
-        <v>851</v>
+        <v>848</v>
       </c>
       <c r="K24" s="9" t="s">
         <v>46</v>
       </c>
       <c r="L24" s="9" t="s">
-        <v>832</v>
+        <v>829</v>
       </c>
     </row>
     <row r="25" spans="1:12" ht="63.75" x14ac:dyDescent="0.45">
@@ -4846,7 +4960,7 @@
         <v>45</v>
       </c>
       <c r="L25" s="9" t="s">
-        <v>832</v>
+        <v>829</v>
       </c>
     </row>
     <row r="26" spans="1:12" ht="153" x14ac:dyDescent="0.45">
@@ -4879,7 +4993,7 @@
       <c r="K26" s="9"/>
       <c r="L26" s="9"/>
     </row>
-    <row r="27" spans="1:12" ht="191.25" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:12" ht="331.5" x14ac:dyDescent="0.45">
       <c r="A27" s="7">
         <v>25</v>
       </c>
@@ -4905,16 +5019,16 @@
         <v>145</v>
       </c>
       <c r="I27" s="14" t="s">
-        <v>852</v>
+        <v>907</v>
       </c>
       <c r="J27" s="14" t="s">
-        <v>853</v>
+        <v>908</v>
       </c>
       <c r="K27" s="9" t="s">
         <v>46</v>
       </c>
       <c r="L27" s="14" t="s">
-        <v>832</v>
+        <v>829</v>
       </c>
     </row>
     <row r="28" spans="1:12" ht="153" x14ac:dyDescent="0.45">
@@ -4943,10 +5057,10 @@
         <v>149</v>
       </c>
       <c r="I28" s="14" t="s">
-        <v>854</v>
+        <v>849</v>
       </c>
       <c r="J28" s="9" t="s">
-        <v>855</v>
+        <v>850</v>
       </c>
       <c r="K28" s="9" t="s">
         <v>45</v>
@@ -4988,7 +5102,7 @@
         <v>46</v>
       </c>
       <c r="L29" s="9" t="s">
-        <v>856</v>
+        <v>851</v>
       </c>
     </row>
     <row r="30" spans="1:12" ht="204" x14ac:dyDescent="0.45">
@@ -5017,16 +5131,16 @@
         <v>157</v>
       </c>
       <c r="I30" s="9" t="s">
-        <v>857</v>
+        <v>852</v>
       </c>
       <c r="J30" s="9" t="s">
-        <v>858</v>
+        <v>853</v>
       </c>
       <c r="K30" s="15" t="s">
         <v>46</v>
       </c>
       <c r="L30" s="9" t="s">
-        <v>832</v>
+        <v>829</v>
       </c>
     </row>
     <row r="31" spans="1:12" ht="102" x14ac:dyDescent="0.45">
@@ -5064,7 +5178,7 @@
         <v>46</v>
       </c>
       <c r="L31" s="9" t="s">
-        <v>859</v>
+        <v>854</v>
       </c>
     </row>
     <row r="32" spans="1:12" ht="178.5" x14ac:dyDescent="0.45">
@@ -5174,7 +5288,7 @@
         <v>45</v>
       </c>
       <c r="L34" s="9" t="s">
-        <v>860</v>
+        <v>855</v>
       </c>
     </row>
     <row r="35" spans="1:12" ht="140.25" x14ac:dyDescent="0.45">
@@ -5203,7 +5317,7 @@
         <v>177</v>
       </c>
       <c r="I35" s="14" t="s">
-        <v>861</v>
+        <v>856</v>
       </c>
       <c r="J35" s="14" t="s">
         <v>815</v>
@@ -5211,8 +5325,8 @@
       <c r="K35" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="L35" s="17" t="s">
-        <v>823</v>
+      <c r="L35" s="14" t="s">
+        <v>874</v>
       </c>
     </row>
     <row r="36" spans="1:12" ht="89.25" x14ac:dyDescent="0.45">
@@ -5241,17 +5355,15 @@
         <v>181</v>
       </c>
       <c r="I36" s="14" t="s">
-        <v>862</v>
+        <v>857</v>
       </c>
       <c r="J36" s="17" t="s">
-        <v>863</v>
+        <v>858</v>
       </c>
       <c r="K36" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="L36" s="17" t="s">
-        <v>823</v>
-      </c>
+      <c r="L36" s="17"/>
     </row>
     <row r="37" spans="1:12" ht="76.5" x14ac:dyDescent="0.45">
       <c r="A37" s="7">
@@ -5277,17 +5389,15 @@
       </c>
       <c r="H37" s="8"/>
       <c r="I37" s="14" t="s">
-        <v>864</v>
+        <v>859</v>
       </c>
       <c r="J37" s="17" t="s">
-        <v>865</v>
+        <v>860</v>
       </c>
       <c r="K37" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="L37" s="17" t="s">
-        <v>823</v>
-      </c>
+      <c r="L37" s="17"/>
     </row>
     <row r="38" spans="1:12" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A38" s="7">
@@ -5459,10 +5569,10 @@
         <v>202</v>
       </c>
       <c r="I42" s="14" t="s">
-        <v>866</v>
+        <v>861</v>
       </c>
       <c r="J42" s="9" t="s">
-        <v>867</v>
+        <v>862</v>
       </c>
       <c r="K42" s="15" t="s">
         <v>46</v>
@@ -5471,7 +5581,7 @@
         <v>823</v>
       </c>
     </row>
-    <row r="43" spans="1:12" ht="140.25" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:12" ht="165.75" x14ac:dyDescent="0.45">
       <c r="A43" s="7">
         <v>41</v>
       </c>
@@ -5496,17 +5606,17 @@
       <c r="H43" s="8" t="s">
         <v>205</v>
       </c>
-      <c r="I43" s="17" t="s">
-        <v>826</v>
-      </c>
-      <c r="J43" s="17" t="s">
-        <v>827</v>
+      <c r="I43" s="14" t="s">
+        <v>909</v>
+      </c>
+      <c r="J43" s="14" t="s">
+        <v>683</v>
       </c>
       <c r="K43" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="L43" s="17" t="s">
-        <v>823</v>
+      <c r="L43" s="14" t="s">
+        <v>910</v>
       </c>
     </row>
     <row r="44" spans="1:12" ht="25.5" x14ac:dyDescent="0.45">
@@ -5540,7 +5650,7 @@
       </c>
       <c r="K44" s="9"/>
       <c r="L44" s="14" t="s">
-        <v>868</v>
+        <v>863</v>
       </c>
     </row>
     <row r="45" spans="1:12" ht="255" x14ac:dyDescent="0.45">
@@ -5569,15 +5679,17 @@
         <v>211</v>
       </c>
       <c r="I45" s="14" t="s">
-        <v>869</v>
+        <v>864</v>
       </c>
       <c r="J45" s="14" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="K45" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="L45" s="9"/>
+      <c r="L45" s="9" t="s">
+        <v>874</v>
+      </c>
     </row>
     <row r="46" spans="1:12" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A46" s="7">
@@ -5613,9 +5725,7 @@
       <c r="K46" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="L46" s="9" t="s">
-        <v>45</v>
-      </c>
+      <c r="L46" s="9"/>
     </row>
     <row r="47" spans="1:12" ht="191.25" x14ac:dyDescent="0.45">
       <c r="A47" s="7">
@@ -5643,19 +5753,19 @@
         <v>218</v>
       </c>
       <c r="I47" s="14" t="s">
-        <v>871</v>
+        <v>866</v>
       </c>
       <c r="J47" s="9" t="s">
-        <v>872</v>
+        <v>867</v>
       </c>
       <c r="K47" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="L47" s="17" t="s">
-        <v>823</v>
-      </c>
-    </row>
-    <row r="48" spans="1:12" ht="102" x14ac:dyDescent="0.45">
+      <c r="L47" s="14" t="s">
+        <v>829</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A48" s="7">
         <v>46</v>
       </c>
@@ -5680,12 +5790,18 @@
       <c r="H48" s="8" t="s">
         <v>222</v>
       </c>
-      <c r="I48" s="9"/>
-      <c r="J48" s="14"/>
+      <c r="I48" s="14" t="s">
+        <v>869</v>
+      </c>
+      <c r="J48" s="14" t="s">
+        <v>815</v>
+      </c>
       <c r="K48" s="9"/>
-      <c r="L48" s="17"/>
-    </row>
-    <row r="49" spans="1:12" ht="178.5" x14ac:dyDescent="0.45">
+      <c r="L48" s="14" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" ht="318.75" x14ac:dyDescent="0.45">
       <c r="A49" s="7">
         <v>47</v>
       </c>
@@ -5710,10 +5826,16 @@
       <c r="H49" s="8" t="s">
         <v>226</v>
       </c>
-      <c r="I49" s="9"/>
-      <c r="J49" s="9"/>
+      <c r="I49" s="14" t="s">
+        <v>870</v>
+      </c>
+      <c r="J49" s="9" t="s">
+        <v>815</v>
+      </c>
       <c r="K49" s="9"/>
-      <c r="L49" s="9"/>
+      <c r="L49" s="9" t="s">
+        <v>829</v>
+      </c>
     </row>
     <row r="50" spans="1:12" ht="280.5" x14ac:dyDescent="0.45">
       <c r="A50" s="7">
@@ -5728,7 +5850,7 @@
       <c r="D50" s="7" t="s">
         <v>228</v>
       </c>
-      <c r="E50" s="7" t="s">
+      <c r="E50" s="13" t="s">
         <v>229</v>
       </c>
       <c r="F50" s="7" t="s">
@@ -5740,10 +5862,16 @@
       <c r="H50" s="8" t="s">
         <v>230</v>
       </c>
-      <c r="I50" s="9"/>
-      <c r="J50" s="9"/>
+      <c r="I50" s="9" t="s">
+        <v>815</v>
+      </c>
+      <c r="J50" s="9" t="s">
+        <v>616</v>
+      </c>
       <c r="K50" s="9"/>
-      <c r="L50" s="9"/>
+      <c r="L50" s="9" t="s">
+        <v>871</v>
+      </c>
     </row>
     <row r="51" spans="1:12" ht="153" x14ac:dyDescent="0.45">
       <c r="A51" s="7">
@@ -5758,7 +5886,7 @@
       <c r="D51" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E51" s="7" t="s">
+      <c r="E51" s="13" t="s">
         <v>233</v>
       </c>
       <c r="F51" s="7" t="s">
@@ -5770,10 +5898,16 @@
       <c r="H51" s="8" t="s">
         <v>234</v>
       </c>
-      <c r="I51" s="9"/>
-      <c r="J51" s="9"/>
+      <c r="I51" s="9" t="s">
+        <v>815</v>
+      </c>
+      <c r="J51" s="14" t="s">
+        <v>872</v>
+      </c>
       <c r="K51" s="9"/>
-      <c r="L51" s="9"/>
+      <c r="L51" s="9" t="s">
+        <v>871</v>
+      </c>
     </row>
     <row r="52" spans="1:12" ht="204" x14ac:dyDescent="0.45">
       <c r="A52" s="7">
@@ -5788,7 +5922,7 @@
       <c r="D52" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="E52" s="7" t="s">
+      <c r="E52" s="13" t="s">
         <v>237</v>
       </c>
       <c r="F52" s="7" t="s">
@@ -5800,10 +5934,16 @@
       <c r="H52" s="8" t="s">
         <v>238</v>
       </c>
-      <c r="I52" s="9"/>
-      <c r="J52" s="9"/>
+      <c r="I52" s="9" t="s">
+        <v>810</v>
+      </c>
+      <c r="J52" s="9" t="s">
+        <v>815</v>
+      </c>
       <c r="K52" s="9"/>
-      <c r="L52" s="9"/>
+      <c r="L52" s="9" t="s">
+        <v>846</v>
+      </c>
     </row>
     <row r="53" spans="1:12" ht="76.5" x14ac:dyDescent="0.45">
       <c r="A53" s="7">
@@ -5818,7 +5958,7 @@
       <c r="D53" s="7" t="s">
         <v>240</v>
       </c>
-      <c r="E53" s="7" t="s">
+      <c r="E53" s="13" t="s">
         <v>241</v>
       </c>
       <c r="F53" s="7" t="s">
@@ -5830,10 +5970,16 @@
       <c r="H53" s="8" t="s">
         <v>242</v>
       </c>
-      <c r="I53" s="9"/>
-      <c r="J53" s="9"/>
+      <c r="I53" s="9" t="s">
+        <v>616</v>
+      </c>
+      <c r="J53" s="9" t="s">
+        <v>815</v>
+      </c>
       <c r="K53" s="9"/>
-      <c r="L53" s="9"/>
+      <c r="L53" s="9" t="s">
+        <v>820</v>
+      </c>
     </row>
     <row r="54" spans="1:12" ht="114.75" x14ac:dyDescent="0.45">
       <c r="A54" s="7">
@@ -5848,7 +5994,7 @@
       <c r="D54" s="7" t="s">
         <v>244</v>
       </c>
-      <c r="E54" s="7" t="s">
+      <c r="E54" s="13" t="s">
         <v>245</v>
       </c>
       <c r="F54" s="7" t="s">
@@ -5860,10 +6006,16 @@
       <c r="H54" s="8" t="s">
         <v>246</v>
       </c>
-      <c r="I54" s="9"/>
-      <c r="J54" s="9"/>
+      <c r="I54" s="9" t="s">
+        <v>815</v>
+      </c>
+      <c r="J54" s="14" t="s">
+        <v>873</v>
+      </c>
       <c r="K54" s="9"/>
-      <c r="L54" s="9"/>
+      <c r="L54" s="9" t="s">
+        <v>874</v>
+      </c>
     </row>
     <row r="55" spans="1:12" ht="89.25" x14ac:dyDescent="0.45">
       <c r="A55" s="7">
@@ -5878,7 +6030,7 @@
       <c r="D55" s="7" t="s">
         <v>247</v>
       </c>
-      <c r="E55" s="7" t="s">
+      <c r="E55" s="13" t="s">
         <v>248</v>
       </c>
       <c r="F55" s="7" t="s">
@@ -5890,10 +6042,16 @@
       <c r="H55" s="8" t="s">
         <v>249</v>
       </c>
-      <c r="I55" s="9"/>
-      <c r="J55" s="9"/>
+      <c r="I55" s="14" t="s">
+        <v>875</v>
+      </c>
+      <c r="J55" s="14" t="s">
+        <v>876</v>
+      </c>
       <c r="K55" s="9"/>
-      <c r="L55" s="9"/>
+      <c r="L55" s="9" t="s">
+        <v>820</v>
+      </c>
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A56" s="7">
@@ -5908,7 +6066,7 @@
       <c r="D56" s="7" t="s">
         <v>251</v>
       </c>
-      <c r="E56" s="7" t="s">
+      <c r="E56" s="13" t="s">
         <v>252</v>
       </c>
       <c r="F56" s="7" t="s">
@@ -5918,12 +6076,18 @@
         <v>46</v>
       </c>
       <c r="H56" s="8"/>
-      <c r="I56" s="9"/>
-      <c r="J56" s="9"/>
+      <c r="I56" s="9" t="s">
+        <v>815</v>
+      </c>
+      <c r="J56" s="9" t="s">
+        <v>815</v>
+      </c>
       <c r="K56" s="9"/>
-      <c r="L56" s="9"/>
-    </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="L56" s="9" t="s">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" ht="51" x14ac:dyDescent="0.45">
       <c r="A57" s="7">
         <v>55</v>
       </c>
@@ -5936,7 +6100,7 @@
       <c r="D57" s="7" t="s">
         <v>254</v>
       </c>
-      <c r="E57" s="7" t="s">
+      <c r="E57" s="13" t="s">
         <v>255</v>
       </c>
       <c r="F57" s="7" t="s">
@@ -5948,10 +6112,16 @@
       <c r="H57" s="8" t="s">
         <v>256</v>
       </c>
-      <c r="I57" s="9"/>
-      <c r="J57" s="9"/>
+      <c r="I57" s="14" t="s">
+        <v>878</v>
+      </c>
+      <c r="J57" s="14" t="s">
+        <v>879</v>
+      </c>
       <c r="K57" s="9"/>
-      <c r="L57" s="9"/>
+      <c r="L57" s="9" t="s">
+        <v>877</v>
+      </c>
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A58" s="7">
@@ -5966,7 +6136,7 @@
       <c r="D58" s="7" t="s">
         <v>257</v>
       </c>
-      <c r="E58" s="7" t="s">
+      <c r="E58" s="13" t="s">
         <v>258</v>
       </c>
       <c r="F58" s="7" t="s">
@@ -5976,8 +6146,12 @@
         <v>46</v>
       </c>
       <c r="H58" s="8"/>
-      <c r="I58" s="9"/>
-      <c r="J58" s="9"/>
+      <c r="I58" s="9" t="s">
+        <v>815</v>
+      </c>
+      <c r="J58" s="9" t="s">
+        <v>815</v>
+      </c>
       <c r="K58" s="9"/>
       <c r="L58" s="9"/>
     </row>
@@ -5994,7 +6168,7 @@
       <c r="D59" s="7" t="s">
         <v>259</v>
       </c>
-      <c r="E59" s="7" t="s">
+      <c r="E59" s="13" t="s">
         <v>260</v>
       </c>
       <c r="F59" s="7" t="s">
@@ -6006,10 +6180,16 @@
       <c r="H59" s="8" t="s">
         <v>261</v>
       </c>
-      <c r="I59" s="9"/>
-      <c r="J59" s="9"/>
+      <c r="I59" s="9" t="s">
+        <v>616</v>
+      </c>
+      <c r="J59" s="9" t="s">
+        <v>815</v>
+      </c>
       <c r="K59" s="9"/>
-      <c r="L59" s="9"/>
+      <c r="L59" s="9" t="s">
+        <v>880</v>
+      </c>
     </row>
     <row r="60" spans="1:12" ht="229.5" x14ac:dyDescent="0.45">
       <c r="A60" s="7">
@@ -6024,7 +6204,7 @@
       <c r="D60" s="7" t="s">
         <v>263</v>
       </c>
-      <c r="E60" s="7" t="s">
+      <c r="E60" s="13" t="s">
         <v>264</v>
       </c>
       <c r="F60" s="7" t="s">
@@ -6036,12 +6216,18 @@
       <c r="H60" s="8" t="s">
         <v>265</v>
       </c>
-      <c r="I60" s="9"/>
-      <c r="J60" s="9"/>
+      <c r="I60" s="14" t="s">
+        <v>881</v>
+      </c>
+      <c r="J60" s="9" t="s">
+        <v>882</v>
+      </c>
       <c r="K60" s="9"/>
-      <c r="L60" s="9"/>
-    </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="L60" s="9" t="s">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" ht="242.25" x14ac:dyDescent="0.45">
       <c r="A61" s="7">
         <v>59</v>
       </c>
@@ -6054,7 +6240,7 @@
       <c r="D61" s="7" t="s">
         <v>267</v>
       </c>
-      <c r="E61" s="7" t="s">
+      <c r="E61" s="13" t="s">
         <v>268</v>
       </c>
       <c r="F61" s="7" t="s">
@@ -6064,10 +6250,16 @@
         <v>46</v>
       </c>
       <c r="H61" s="8"/>
-      <c r="I61" s="9"/>
-      <c r="J61" s="9"/>
+      <c r="I61" s="14" t="s">
+        <v>883</v>
+      </c>
+      <c r="J61" s="9" t="s">
+        <v>884</v>
+      </c>
       <c r="K61" s="9"/>
-      <c r="L61" s="9"/>
+      <c r="L61" s="9" t="s">
+        <v>885</v>
+      </c>
     </row>
     <row r="62" spans="1:12" ht="242.25" x14ac:dyDescent="0.45">
       <c r="A62" s="7">
@@ -6082,7 +6274,7 @@
       <c r="D62" s="7" t="s">
         <v>270</v>
       </c>
-      <c r="E62" s="7" t="s">
+      <c r="E62" s="13" t="s">
         <v>271</v>
       </c>
       <c r="F62" s="7" t="s">
@@ -6094,10 +6286,16 @@
       <c r="H62" s="8" t="s">
         <v>272</v>
       </c>
-      <c r="I62" s="9"/>
-      <c r="J62" s="9"/>
+      <c r="I62" s="9" t="s">
+        <v>627</v>
+      </c>
+      <c r="J62" s="9" t="s">
+        <v>616</v>
+      </c>
       <c r="K62" s="9"/>
-      <c r="L62" s="9"/>
+      <c r="L62" s="9" t="s">
+        <v>880</v>
+      </c>
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A63" s="7">
@@ -6112,7 +6310,7 @@
       <c r="D63" s="7" t="s">
         <v>274</v>
       </c>
-      <c r="E63" s="7" t="s">
+      <c r="E63" s="13" t="s">
         <v>275</v>
       </c>
       <c r="F63" s="7" t="s">
@@ -6122,12 +6320,18 @@
         <v>46</v>
       </c>
       <c r="H63" s="8"/>
-      <c r="I63" s="9"/>
-      <c r="J63" s="9"/>
+      <c r="I63" s="9" t="s">
+        <v>815</v>
+      </c>
+      <c r="J63" s="9" t="s">
+        <v>815</v>
+      </c>
       <c r="K63" s="9"/>
-      <c r="L63" s="9"/>
-    </row>
-    <row r="64" spans="1:12" ht="165.75" x14ac:dyDescent="0.45">
+      <c r="L63" s="9" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" ht="178.5" x14ac:dyDescent="0.45">
       <c r="A64" s="7">
         <v>62</v>
       </c>
@@ -6140,7 +6344,7 @@
       <c r="D64" s="7" t="s">
         <v>277</v>
       </c>
-      <c r="E64" s="7" t="s">
+      <c r="E64" s="13" t="s">
         <v>278</v>
       </c>
       <c r="F64" s="7" t="s">
@@ -6152,10 +6356,16 @@
       <c r="H64" s="8" t="s">
         <v>279</v>
       </c>
-      <c r="I64" s="9"/>
-      <c r="J64" s="9"/>
+      <c r="I64" s="14" t="s">
+        <v>886</v>
+      </c>
+      <c r="J64" s="9" t="s">
+        <v>815</v>
+      </c>
       <c r="K64" s="9"/>
-      <c r="L64" s="9"/>
+      <c r="L64" s="9" t="s">
+        <v>874</v>
+      </c>
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A65" s="7">
@@ -6170,7 +6380,7 @@
       <c r="D65" s="7" t="s">
         <v>281</v>
       </c>
-      <c r="E65" s="7" t="s">
+      <c r="E65" s="13" t="s">
         <v>282</v>
       </c>
       <c r="F65" s="7" t="s">
@@ -6180,12 +6390,18 @@
         <v>46</v>
       </c>
       <c r="H65" s="8"/>
-      <c r="I65" s="9"/>
-      <c r="J65" s="9"/>
+      <c r="I65" s="9" t="s">
+        <v>815</v>
+      </c>
+      <c r="J65" s="9" t="s">
+        <v>815</v>
+      </c>
       <c r="K65" s="9"/>
-      <c r="L65" s="9"/>
-    </row>
-    <row r="66" spans="1:12" ht="102" x14ac:dyDescent="0.45">
+      <c r="L65" s="9" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12" ht="382.5" x14ac:dyDescent="0.45">
       <c r="A66" s="7">
         <v>64</v>
       </c>
@@ -6198,7 +6414,7 @@
       <c r="D66" s="7" t="s">
         <v>284</v>
       </c>
-      <c r="E66" s="7" t="s">
+      <c r="E66" s="13" t="s">
         <v>285</v>
       </c>
       <c r="F66" s="7" t="s">
@@ -6210,10 +6426,16 @@
       <c r="H66" s="8" t="s">
         <v>286</v>
       </c>
-      <c r="I66" s="9"/>
-      <c r="J66" s="9"/>
+      <c r="I66" s="14" t="s">
+        <v>887</v>
+      </c>
+      <c r="J66" s="14" t="s">
+        <v>888</v>
+      </c>
       <c r="K66" s="9"/>
-      <c r="L66" s="9"/>
+      <c r="L66" s="9" t="s">
+        <v>874</v>
+      </c>
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A67" s="7">
@@ -6228,7 +6450,7 @@
       <c r="D67" s="7" t="s">
         <v>287</v>
       </c>
-      <c r="E67" s="7" t="s">
+      <c r="E67" s="13" t="s">
         <v>288</v>
       </c>
       <c r="F67" s="7" t="s">
@@ -6238,10 +6460,16 @@
         <v>46</v>
       </c>
       <c r="H67" s="8"/>
-      <c r="I67" s="9"/>
-      <c r="J67" s="9"/>
+      <c r="I67" s="9" t="s">
+        <v>815</v>
+      </c>
+      <c r="J67" s="9" t="s">
+        <v>815</v>
+      </c>
       <c r="K67" s="9"/>
-      <c r="L67" s="9"/>
+      <c r="L67" s="9" t="s">
+        <v>885</v>
+      </c>
     </row>
     <row r="68" spans="1:12" ht="140.25" x14ac:dyDescent="0.45">
       <c r="A68" s="7">
@@ -6256,7 +6484,7 @@
       <c r="D68" s="7" t="s">
         <v>289</v>
       </c>
-      <c r="E68" s="7" t="s">
+      <c r="E68" s="13" t="s">
         <v>290</v>
       </c>
       <c r="F68" s="7" t="s">
@@ -6268,12 +6496,18 @@
       <c r="H68" s="8" t="s">
         <v>291</v>
       </c>
-      <c r="I68" s="9"/>
-      <c r="J68" s="9"/>
+      <c r="I68" s="9" t="s">
+        <v>815</v>
+      </c>
+      <c r="J68" s="9" t="s">
+        <v>815</v>
+      </c>
       <c r="K68" s="9"/>
-      <c r="L68" s="9"/>
-    </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="L68" s="9" t="s">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12" ht="344.25" x14ac:dyDescent="0.45">
       <c r="A69" s="7">
         <v>67</v>
       </c>
@@ -6286,7 +6520,7 @@
       <c r="D69" s="7" t="s">
         <v>292</v>
       </c>
-      <c r="E69" s="7" t="s">
+      <c r="E69" s="13" t="s">
         <v>293</v>
       </c>
       <c r="F69" s="7" t="s">
@@ -6296,10 +6530,16 @@
         <v>46</v>
       </c>
       <c r="H69" s="8"/>
-      <c r="I69" s="9"/>
-      <c r="J69" s="9"/>
+      <c r="I69" s="14" t="s">
+        <v>889</v>
+      </c>
+      <c r="J69" s="14" t="s">
+        <v>890</v>
+      </c>
       <c r="K69" s="9"/>
-      <c r="L69" s="9"/>
+      <c r="L69" s="9" t="s">
+        <v>885</v>
+      </c>
     </row>
     <row r="70" spans="1:12" ht="114.75" x14ac:dyDescent="0.45">
       <c r="A70" s="7">
@@ -6314,7 +6554,7 @@
       <c r="D70" s="7" t="s">
         <v>295</v>
       </c>
-      <c r="E70" s="7" t="s">
+      <c r="E70" s="13" t="s">
         <v>296</v>
       </c>
       <c r="F70" s="7" t="s">
@@ -6326,12 +6566,18 @@
       <c r="H70" s="8" t="s">
         <v>297</v>
       </c>
-      <c r="I70" s="9"/>
-      <c r="J70" s="9"/>
+      <c r="I70" s="14" t="s">
+        <v>891</v>
+      </c>
+      <c r="J70" s="9" t="s">
+        <v>815</v>
+      </c>
       <c r="K70" s="9"/>
-      <c r="L70" s="9"/>
-    </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="L70" s="9" t="s">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12" ht="51" x14ac:dyDescent="0.45">
       <c r="A71" s="7">
         <v>69</v>
       </c>
@@ -6344,7 +6590,7 @@
       <c r="D71" s="7" t="s">
         <v>299</v>
       </c>
-      <c r="E71" s="7" t="s">
+      <c r="E71" s="13" t="s">
         <v>300</v>
       </c>
       <c r="F71" s="7" t="s">
@@ -6354,10 +6600,16 @@
         <v>46</v>
       </c>
       <c r="H71" s="8"/>
-      <c r="I71" s="9"/>
-      <c r="J71" s="9"/>
+      <c r="I71" s="14" t="s">
+        <v>892</v>
+      </c>
+      <c r="J71" s="14" t="s">
+        <v>893</v>
+      </c>
       <c r="K71" s="9"/>
-      <c r="L71" s="9"/>
+      <c r="L71" s="9" t="s">
+        <v>877</v>
+      </c>
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A72" s="7">
@@ -6372,7 +6624,7 @@
       <c r="D72" s="7" t="s">
         <v>301</v>
       </c>
-      <c r="E72" s="7" t="s">
+      <c r="E72" s="13" t="s">
         <v>302</v>
       </c>
       <c r="F72" s="7" t="s">
@@ -6382,12 +6634,18 @@
         <v>46</v>
       </c>
       <c r="H72" s="8"/>
-      <c r="I72" s="9"/>
-      <c r="J72" s="9"/>
+      <c r="I72" s="9" t="s">
+        <v>815</v>
+      </c>
+      <c r="J72" s="9" t="s">
+        <v>815</v>
+      </c>
       <c r="K72" s="9"/>
-      <c r="L72" s="9"/>
-    </row>
-    <row r="73" spans="1:12" ht="89.25" x14ac:dyDescent="0.45">
+      <c r="L72" s="9" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12" ht="140.25" x14ac:dyDescent="0.45">
       <c r="A73" s="7">
         <v>71</v>
       </c>
@@ -6400,7 +6658,7 @@
       <c r="D73" s="7" t="s">
         <v>304</v>
       </c>
-      <c r="E73" s="7" t="s">
+      <c r="E73" s="13" t="s">
         <v>305</v>
       </c>
       <c r="F73" s="7" t="s">
@@ -6412,12 +6670,18 @@
       <c r="H73" s="8" t="s">
         <v>306</v>
       </c>
-      <c r="I73" s="9"/>
-      <c r="J73" s="9"/>
+      <c r="I73" s="14" t="s">
+        <v>894</v>
+      </c>
+      <c r="J73" s="9" t="s">
+        <v>815</v>
+      </c>
       <c r="K73" s="9"/>
-      <c r="L73" s="9"/>
-    </row>
-    <row r="74" spans="1:12" ht="140.25" x14ac:dyDescent="0.45">
+      <c r="L73" s="9" t="s">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="74" spans="1:12" ht="191.25" x14ac:dyDescent="0.45">
       <c r="A74" s="7">
         <v>72</v>
       </c>
@@ -6430,7 +6694,7 @@
       <c r="D74" s="7" t="s">
         <v>308</v>
       </c>
-      <c r="E74" s="7" t="s">
+      <c r="E74" s="13" t="s">
         <v>309</v>
       </c>
       <c r="F74" s="7" t="s">
@@ -6442,10 +6706,16 @@
       <c r="H74" s="8" t="s">
         <v>310</v>
       </c>
-      <c r="I74" s="9"/>
-      <c r="J74" s="9"/>
+      <c r="I74" s="14" t="s">
+        <v>895</v>
+      </c>
+      <c r="J74" s="9" t="s">
+        <v>815</v>
+      </c>
       <c r="K74" s="9"/>
-      <c r="L74" s="9"/>
+      <c r="L74" s="9" t="s">
+        <v>874</v>
+      </c>
     </row>
     <row r="75" spans="1:12" ht="216.75" x14ac:dyDescent="0.45">
       <c r="A75" s="7">
@@ -6460,7 +6730,7 @@
       <c r="D75" s="7" t="s">
         <v>312</v>
       </c>
-      <c r="E75" s="7" t="s">
+      <c r="E75" s="13" t="s">
         <v>313</v>
       </c>
       <c r="F75" s="7" t="s">
@@ -6472,10 +6742,16 @@
       <c r="H75" s="8" t="s">
         <v>314</v>
       </c>
-      <c r="I75" s="9"/>
-      <c r="J75" s="9"/>
+      <c r="I75" s="9" t="s">
+        <v>897</v>
+      </c>
+      <c r="J75" s="14" t="s">
+        <v>898</v>
+      </c>
       <c r="K75" s="9"/>
-      <c r="L75" s="9"/>
+      <c r="L75" s="9" t="s">
+        <v>896</v>
+      </c>
     </row>
     <row r="76" spans="1:12" ht="204" x14ac:dyDescent="0.45">
       <c r="A76" s="7">
@@ -6490,7 +6766,7 @@
       <c r="D76" s="7" t="s">
         <v>316</v>
       </c>
-      <c r="E76" s="7" t="s">
+      <c r="E76" s="13" t="s">
         <v>317</v>
       </c>
       <c r="F76" s="7" t="s">
@@ -6502,10 +6778,16 @@
       <c r="H76" s="8" t="s">
         <v>318</v>
       </c>
-      <c r="I76" s="9"/>
-      <c r="J76" s="9"/>
+      <c r="I76" s="9" t="s">
+        <v>815</v>
+      </c>
+      <c r="J76" s="9" t="s">
+        <v>815</v>
+      </c>
       <c r="K76" s="9"/>
-      <c r="L76" s="9"/>
+      <c r="L76" s="9" t="s">
+        <v>880</v>
+      </c>
     </row>
     <row r="77" spans="1:12" ht="140.25" x14ac:dyDescent="0.45">
       <c r="A77" s="7">
@@ -6520,7 +6802,7 @@
       <c r="D77" s="7" t="s">
         <v>320</v>
       </c>
-      <c r="E77" s="7" t="s">
+      <c r="E77" s="13" t="s">
         <v>321</v>
       </c>
       <c r="F77" s="7" t="s">
@@ -6532,12 +6814,18 @@
       <c r="H77" s="8" t="s">
         <v>322</v>
       </c>
-      <c r="I77" s="9"/>
-      <c r="J77" s="9"/>
+      <c r="I77" s="14" t="s">
+        <v>900</v>
+      </c>
+      <c r="J77" s="9" t="s">
+        <v>901</v>
+      </c>
       <c r="K77" s="9"/>
-      <c r="L77" s="9"/>
-    </row>
-    <row r="78" spans="1:12" ht="102" x14ac:dyDescent="0.45">
+      <c r="L77" s="9" t="s">
+        <v>899</v>
+      </c>
+    </row>
+    <row r="78" spans="1:12" ht="357" x14ac:dyDescent="0.45">
       <c r="A78" s="7">
         <v>76</v>
       </c>
@@ -6550,7 +6838,7 @@
       <c r="D78" s="7" t="s">
         <v>324</v>
       </c>
-      <c r="E78" s="7" t="s">
+      <c r="E78" s="13" t="s">
         <v>325</v>
       </c>
       <c r="F78" s="7" t="s">
@@ -6562,10 +6850,16 @@
       <c r="H78" s="8" t="s">
         <v>326</v>
       </c>
-      <c r="I78" s="9"/>
-      <c r="J78" s="9"/>
+      <c r="I78" s="14" t="s">
+        <v>902</v>
+      </c>
+      <c r="J78" s="14" t="s">
+        <v>903</v>
+      </c>
       <c r="K78" s="9"/>
-      <c r="L78" s="9"/>
+      <c r="L78" s="9" t="s">
+        <v>874</v>
+      </c>
     </row>
     <row r="79" spans="1:12" ht="165.75" x14ac:dyDescent="0.45">
       <c r="A79" s="7">
@@ -6580,7 +6874,7 @@
       <c r="D79" s="7" t="s">
         <v>328</v>
       </c>
-      <c r="E79" s="7" t="s">
+      <c r="E79" s="13" t="s">
         <v>329</v>
       </c>
       <c r="F79" s="7" t="s">
@@ -6592,10 +6886,16 @@
       <c r="H79" s="8" t="s">
         <v>330</v>
       </c>
-      <c r="I79" s="9"/>
-      <c r="J79" s="9"/>
+      <c r="I79" s="14" t="s">
+        <v>904</v>
+      </c>
+      <c r="J79" s="9" t="s">
+        <v>815</v>
+      </c>
       <c r="K79" s="9"/>
-      <c r="L79" s="9"/>
+      <c r="L79" s="9" t="s">
+        <v>874</v>
+      </c>
     </row>
     <row r="80" spans="1:12" ht="89.25" x14ac:dyDescent="0.45">
       <c r="A80" s="7">
@@ -6610,7 +6910,7 @@
       <c r="D80" s="7" t="s">
         <v>332</v>
       </c>
-      <c r="E80" s="7" t="s">
+      <c r="E80" s="13" t="s">
         <v>333</v>
       </c>
       <c r="F80" s="7" t="s">
@@ -6622,10 +6922,16 @@
       <c r="H80" s="8" t="s">
         <v>334</v>
       </c>
-      <c r="I80" s="9"/>
-      <c r="J80" s="9"/>
+      <c r="I80" s="9" t="s">
+        <v>815</v>
+      </c>
+      <c r="J80" s="9" t="s">
+        <v>815</v>
+      </c>
       <c r="K80" s="9"/>
-      <c r="L80" s="9"/>
+      <c r="L80" s="9" t="s">
+        <v>885</v>
+      </c>
     </row>
     <row r="81" spans="1:12" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A81" s="7">
@@ -6640,7 +6946,7 @@
       <c r="D81" s="7" t="s">
         <v>335</v>
       </c>
-      <c r="E81" s="7" t="s">
+      <c r="E81" s="13" t="s">
         <v>336</v>
       </c>
       <c r="F81" s="7" t="s">
@@ -6652,10 +6958,16 @@
       <c r="H81" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="I81" s="9"/>
-      <c r="J81" s="9"/>
+      <c r="I81" s="9" t="s">
+        <v>625</v>
+      </c>
+      <c r="J81" s="9" t="s">
+        <v>815</v>
+      </c>
       <c r="K81" s="9"/>
-      <c r="L81" s="9"/>
+      <c r="L81" s="9" t="s">
+        <v>877</v>
+      </c>
     </row>
     <row r="82" spans="1:12" ht="204" x14ac:dyDescent="0.45">
       <c r="A82" s="7">
@@ -8817,9 +9129,41 @@
     <hyperlink ref="E49" r:id="rId46" xr:uid="{1C8774A2-A9A1-4F43-98F6-C951B8423B16}"/>
     <hyperlink ref="E4" r:id="rId47" xr:uid="{E8146D32-CBAE-417B-AA12-BA90E9334704}"/>
     <hyperlink ref="E44" r:id="rId48" xr:uid="{2F1D026A-CF24-42C1-B8D0-B911D595C828}"/>
+    <hyperlink ref="E50" r:id="rId49" xr:uid="{CBEA990E-3760-41AA-976E-32461EACF251}"/>
+    <hyperlink ref="E51" r:id="rId50" xr:uid="{2A95B796-AFE1-4454-A10E-11C2643B0426}"/>
+    <hyperlink ref="E52" r:id="rId51" xr:uid="{56C84C87-C464-4F83-9AF2-C7B6DDC3C935}"/>
+    <hyperlink ref="E53" r:id="rId52" xr:uid="{7F09C477-C202-4B94-92EC-36EDBC6D9E27}"/>
+    <hyperlink ref="E54" r:id="rId53" xr:uid="{FD8CEE68-A9FD-4C5A-A628-B13980DF6DE7}"/>
+    <hyperlink ref="E55" r:id="rId54" xr:uid="{0A030746-C3B4-420C-81DA-4945CB82B84C}"/>
+    <hyperlink ref="E56" r:id="rId55" xr:uid="{CE28EC2B-75F6-4DBC-946E-6ECB03E548C0}"/>
+    <hyperlink ref="E57" r:id="rId56" xr:uid="{7FEC93AA-E64E-4472-9649-EA39B1C02F48}"/>
+    <hyperlink ref="E58" r:id="rId57" xr:uid="{E9777CCF-1C79-42FA-879F-F67F0968955D}"/>
+    <hyperlink ref="E59" r:id="rId58" xr:uid="{6BC495F2-D2D5-421E-9441-DFC89F0878BD}"/>
+    <hyperlink ref="E60" r:id="rId59" xr:uid="{2AB4E712-0C4F-4BF3-8E95-622CCA457C99}"/>
+    <hyperlink ref="E61" r:id="rId60" xr:uid="{D79AAE37-0CE4-4609-8362-F0C96E6BE97F}"/>
+    <hyperlink ref="E62" r:id="rId61" xr:uid="{0BDF392A-DDCB-42C0-AAA6-C07D9EB666DA}"/>
+    <hyperlink ref="E63" r:id="rId62" xr:uid="{F8DC553C-18EA-4338-8AED-65EF3448BB37}"/>
+    <hyperlink ref="E64" r:id="rId63" xr:uid="{5E6C98BF-B863-4E72-BF73-C93E2F5B5ACA}"/>
+    <hyperlink ref="E65" r:id="rId64" xr:uid="{5A007684-3A93-4E09-BF32-87C4D90920D5}"/>
+    <hyperlink ref="E66" r:id="rId65" xr:uid="{DC99492A-B459-483F-A6EA-4E9D0AB281BF}"/>
+    <hyperlink ref="E67" r:id="rId66" xr:uid="{BF0339BC-8F76-4158-BC62-089AAC1BF713}"/>
+    <hyperlink ref="E68" r:id="rId67" xr:uid="{B831444B-8F34-44C0-B7F5-4B21A3C18178}"/>
+    <hyperlink ref="E69" r:id="rId68" xr:uid="{D1ACEAAB-9EBA-4851-9837-4B3A64772FAE}"/>
+    <hyperlink ref="E70" r:id="rId69" xr:uid="{B75B6CCB-A4FD-4A19-9544-6E96E487D118}"/>
+    <hyperlink ref="E71" r:id="rId70" xr:uid="{3DD7E24A-7964-40E2-9A03-11731A0BF316}"/>
+    <hyperlink ref="E72" r:id="rId71" xr:uid="{815190F0-1FBE-4243-ABD5-950942ABC225}"/>
+    <hyperlink ref="E73" r:id="rId72" xr:uid="{1B32984C-52FE-4481-978E-07409B1FC0B6}"/>
+    <hyperlink ref="E74" r:id="rId73" xr:uid="{FCDC2AC8-B62D-4F24-936D-5D8A1B3C486F}"/>
+    <hyperlink ref="E75" r:id="rId74" xr:uid="{F74AD02E-6932-49CB-8D15-3F9BE7B6FAD5}"/>
+    <hyperlink ref="E76" r:id="rId75" xr:uid="{6DB0FBC1-A2FC-4992-8D02-88D1146D9E5B}"/>
+    <hyperlink ref="E77" r:id="rId76" xr:uid="{08CFB285-B096-4860-8D26-DE2357BBFF10}"/>
+    <hyperlink ref="E78" r:id="rId77" xr:uid="{72C08F11-BD1C-4FC1-8FC6-A3ECAB5821B7}"/>
+    <hyperlink ref="E79" r:id="rId78" xr:uid="{E634947A-3983-43B6-A09F-EEF76ECA103B}"/>
+    <hyperlink ref="E80" r:id="rId79" xr:uid="{BC84FC9C-B026-4647-A05F-196336FD71D2}"/>
+    <hyperlink ref="E81" r:id="rId80" xr:uid="{91A7A9B8-AE96-45BF-A966-E53E2DDD1021}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId49"/>
+  <pageSetup orientation="portrait" r:id="rId81"/>
 </worksheet>
 </file>
 
@@ -9416,7 +9760,7 @@
         <v>718</v>
       </c>
       <c r="C42" s="16" t="s">
-        <v>828</v>
+        <v>826</v>
       </c>
       <c r="D42" s="11" t="s">
         <v>719</v>

</xml_diff>